<commit_message>
Update: Added new features/fixes
</commit_message>
<xml_diff>
--- a/hostel_backend/HOSTEL PONNI.xlsx
+++ b/hostel_backend/HOSTEL PONNI.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D7738D-2F5F-4F64-9EB5-99CFDBD8E0A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6AB3F9C-E76D-438C-8EE4-5313D8D68F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4579,7 +4579,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4601,6 +4601,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4648,7 +4654,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4698,6 +4704,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5638,29 +5647,29 @@
       <c r="A15" s="6">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="B15" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7" t="s">
+      <c r="D15" s="18"/>
+      <c r="E15" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="18"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
       <c r="O15" s="4"/>
@@ -5680,31 +5689,31 @@
       <c r="A16" s="6">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="4" t="s">
+      <c r="B16" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7" t="s">
+      <c r="D16" s="18"/>
+      <c r="E16" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="18"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
       <c r="O16" s="4"/>
@@ -11374,26 +11383,26 @@
       <c r="A136" s="6">
         <v>135</v>
       </c>
-      <c r="B136" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C136" s="4" t="s">
+      <c r="B136" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C136" s="18" t="s">
         <v>284</v>
       </c>
-      <c r="D136" s="7"/>
-      <c r="E136" s="7" t="s">
+      <c r="D136" s="18"/>
+      <c r="E136" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F136" s="7" t="s">
+      <c r="F136" s="18" t="s">
         <v>264</v>
       </c>
-      <c r="G136" s="7" t="s">
+      <c r="G136" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H136" s="7" t="s">
+      <c r="H136" s="18" t="s">
         <v>283</v>
       </c>
-      <c r="I136" s="7"/>
+      <c r="I136" s="18"/>
       <c r="J136" s="7"/>
       <c r="K136" s="7"/>
       <c r="L136" s="7"/>
@@ -12044,26 +12053,26 @@
       <c r="A151" s="6">
         <v>150</v>
       </c>
-      <c r="B151" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C151" s="4" t="s">
+      <c r="B151" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C151" s="18" t="s">
         <v>318</v>
       </c>
-      <c r="D151" s="7"/>
-      <c r="E151" s="7" t="s">
+      <c r="D151" s="18"/>
+      <c r="E151" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F151" s="7" t="s">
+      <c r="F151" s="18" t="s">
         <v>314</v>
       </c>
-      <c r="G151" s="7" t="s">
+      <c r="G151" s="18" t="s">
         <v>307</v>
       </c>
-      <c r="H151" s="7" t="s">
+      <c r="H151" s="18" t="s">
         <v>315</v>
       </c>
-      <c r="I151" s="7" t="s">
+      <c r="I151" s="18" t="s">
         <v>295</v>
       </c>
       <c r="J151" s="7"/>
@@ -12272,26 +12281,26 @@
       <c r="A156" s="6">
         <v>155</v>
       </c>
-      <c r="B156" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C156" s="4" t="s">
+      <c r="B156" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C156" s="18" t="s">
         <v>326</v>
       </c>
-      <c r="D156" s="7"/>
-      <c r="E156" s="7" t="s">
+      <c r="D156" s="18"/>
+      <c r="E156" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F156" s="7" t="s">
+      <c r="F156" s="18" t="s">
         <v>327</v>
       </c>
-      <c r="G156" s="7" t="s">
+      <c r="G156" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H156" s="7" t="s">
+      <c r="H156" s="18" t="s">
         <v>328</v>
       </c>
-      <c r="I156" s="7" t="s">
+      <c r="I156" s="18" t="s">
         <v>107</v>
       </c>
       <c r="J156" s="7"/>
@@ -12316,26 +12325,26 @@
       <c r="A157" s="6">
         <v>156</v>
       </c>
-      <c r="B157" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C157" s="4" t="s">
+      <c r="B157" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C157" s="18" t="s">
         <v>329</v>
       </c>
-      <c r="D157" s="7"/>
-      <c r="E157" s="7" t="s">
+      <c r="D157" s="18"/>
+      <c r="E157" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F157" s="7" t="s">
+      <c r="F157" s="18" t="s">
         <v>330</v>
       </c>
-      <c r="G157" s="7" t="s">
+      <c r="G157" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H157" s="7" t="s">
+      <c r="H157" s="18" t="s">
         <v>328</v>
       </c>
-      <c r="I157" s="7" t="s">
+      <c r="I157" s="18" t="s">
         <v>291</v>
       </c>
       <c r="J157" s="7"/>
@@ -12360,26 +12369,26 @@
       <c r="A158" s="6">
         <v>157</v>
       </c>
-      <c r="B158" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C158" s="4" t="s">
+      <c r="B158" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C158" s="18" t="s">
         <v>331</v>
       </c>
-      <c r="D158" s="7"/>
-      <c r="E158" s="7" t="s">
+      <c r="D158" s="18"/>
+      <c r="E158" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F158" s="7" t="s">
+      <c r="F158" s="18" t="s">
         <v>304</v>
       </c>
-      <c r="G158" s="7" t="s">
+      <c r="G158" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H158" s="7" t="s">
+      <c r="H158" s="18" t="s">
         <v>328</v>
       </c>
-      <c r="I158" s="7" t="s">
+      <c r="I158" s="18" t="s">
         <v>198</v>
       </c>
       <c r="J158" s="7"/>
@@ -12404,26 +12413,26 @@
       <c r="A159" s="6">
         <v>158</v>
       </c>
-      <c r="B159" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C159" s="4" t="s">
+      <c r="B159" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C159" s="18" t="s">
         <v>332</v>
       </c>
-      <c r="D159" s="7"/>
-      <c r="E159" s="7" t="s">
+      <c r="D159" s="18"/>
+      <c r="E159" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F159" s="7" t="s">
+      <c r="F159" s="18" t="s">
         <v>264</v>
       </c>
-      <c r="G159" s="7" t="s">
+      <c r="G159" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H159" s="7" t="s">
+      <c r="H159" s="18" t="s">
         <v>328</v>
       </c>
-      <c r="I159" s="7" t="s">
+      <c r="I159" s="18" t="s">
         <v>295</v>
       </c>
       <c r="J159" s="7"/>
@@ -12488,26 +12497,26 @@
       <c r="A161" s="6">
         <v>160</v>
       </c>
-      <c r="B161" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C161" s="4" t="s">
+      <c r="B161" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C161" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="D161" s="7"/>
-      <c r="E161" s="7" t="s">
+      <c r="D161" s="18"/>
+      <c r="E161" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F161" s="7" t="s">
+      <c r="F161" s="18" t="s">
         <v>335</v>
       </c>
-      <c r="G161" s="7" t="s">
+      <c r="G161" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H161" s="7" t="s">
+      <c r="H161" s="18" t="s">
         <v>333</v>
       </c>
-      <c r="I161" s="7" t="s">
+      <c r="I161" s="18" t="s">
         <v>336</v>
       </c>
       <c r="J161" s="7"/>
@@ -12706,26 +12715,26 @@
       <c r="A166" s="6">
         <v>165</v>
       </c>
-      <c r="B166" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C166" s="4" t="s">
+      <c r="B166" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C166" s="18" t="s">
         <v>341</v>
       </c>
-      <c r="D166" s="7"/>
-      <c r="E166" s="7" t="s">
+      <c r="D166" s="18"/>
+      <c r="E166" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F166" s="7" t="s">
+      <c r="F166" s="18" t="s">
         <v>264</v>
       </c>
-      <c r="G166" s="7" t="s">
+      <c r="G166" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H166" s="7" t="s">
+      <c r="H166" s="18" t="s">
         <v>338</v>
       </c>
-      <c r="I166" s="7" t="s">
+      <c r="I166" s="18" t="s">
         <v>251</v>
       </c>
       <c r="J166" s="7"/>
@@ -12750,26 +12759,26 @@
       <c r="A167" s="6">
         <v>166</v>
       </c>
-      <c r="B167" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C167" s="4" t="s">
+      <c r="B167" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C167" s="18" t="s">
         <v>342</v>
       </c>
-      <c r="D167" s="7"/>
-      <c r="E167" s="7" t="s">
+      <c r="D167" s="18"/>
+      <c r="E167" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F167" s="7" t="s">
+      <c r="F167" s="18" t="s">
         <v>264</v>
       </c>
-      <c r="G167" s="7" t="s">
+      <c r="G167" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H167" s="7" t="s">
+      <c r="H167" s="18" t="s">
         <v>338</v>
       </c>
-      <c r="I167" s="7" t="s">
+      <c r="I167" s="18" t="s">
         <v>61</v>
       </c>
       <c r="J167" s="7"/>
@@ -12794,26 +12803,26 @@
       <c r="A168" s="6">
         <v>167</v>
       </c>
-      <c r="B168" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C168" s="4" t="s">
+      <c r="B168" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C168" s="18" t="s">
         <v>343</v>
       </c>
-      <c r="D168" s="7"/>
-      <c r="E168" s="7" t="s">
+      <c r="D168" s="18"/>
+      <c r="E168" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F168" s="7" t="s">
+      <c r="F168" s="18" t="s">
         <v>344</v>
       </c>
-      <c r="G168" s="7" t="s">
+      <c r="G168" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H168" s="7" t="s">
+      <c r="H168" s="18" t="s">
         <v>345</v>
       </c>
-      <c r="I168" s="7" t="s">
+      <c r="I168" s="18" t="s">
         <v>186</v>
       </c>
       <c r="J168" s="7"/>
@@ -12838,26 +12847,26 @@
       <c r="A169" s="6">
         <v>168</v>
       </c>
-      <c r="B169" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C169" s="4" t="s">
+      <c r="B169" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C169" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="D169" s="7"/>
-      <c r="E169" s="7" t="s">
+      <c r="D169" s="18"/>
+      <c r="E169" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F169" s="7" t="s">
+      <c r="F169" s="18" t="s">
         <v>347</v>
       </c>
-      <c r="G169" s="7" t="s">
+      <c r="G169" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H169" s="7" t="s">
+      <c r="H169" s="18" t="s">
         <v>345</v>
       </c>
-      <c r="I169" s="7" t="s">
+      <c r="I169" s="18" t="s">
         <v>232</v>
       </c>
       <c r="J169" s="7"/>
@@ -12882,26 +12891,26 @@
       <c r="A170" s="6">
         <v>169</v>
       </c>
-      <c r="B170" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C170" s="4" t="s">
+      <c r="B170" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C170" s="18" t="s">
         <v>348</v>
       </c>
-      <c r="D170" s="7"/>
-      <c r="E170" s="7" t="s">
+      <c r="D170" s="18"/>
+      <c r="E170" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="F170" s="7" t="s">
+      <c r="F170" s="18" t="s">
         <v>349</v>
       </c>
-      <c r="G170" s="7" t="s">
+      <c r="G170" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="H170" s="7" t="s">
+      <c r="H170" s="18" t="s">
         <v>345</v>
       </c>
-      <c r="I170" s="7" t="s">
+      <c r="I170" s="18" t="s">
         <v>350</v>
       </c>
       <c r="J170" s="7"/>

</xml_diff>